<commit_message>
updated xlsx and r script
Updated changes to xlsx and r script
</commit_message>
<xml_diff>
--- a/data/metaB_effort.xlsx
+++ b/data/metaB_effort.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/colleen_keefer_fws_gov/Documents/Desktop/Automation tool github/Implementation_Planning/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EB76DA9-E943-4AE9-872A-200D5C95EC43}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B75EAC9-2852-43B1-B438-69C1300C3AEC}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2835" windowWidth="29040" windowHeight="15720" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
+    <workbookView xWindow="1836" yWindow="3552" windowWidth="22980" windowHeight="11616" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
   </bookViews>
   <sheets>
     <sheet name="metaB_effort" sheetId="1" r:id="rId1"/>
@@ -1229,7 +1229,7 @@
         <v>12</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I7">
         <v>20</v>
@@ -1606,6 +1606,9 @@
       </c>
       <c r="G21" t="s">
         <v>28</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
       </c>
       <c r="I21">
         <v>10</v>

</xml_diff>

<commit_message>
Updated Table and Figure for 2025 Partner Planning Document
</commit_message>
<xml_diff>
--- a/data/metaB_effort.xlsx
+++ b/data/metaB_effort.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/colleen_keefer_fws_gov/Documents/Desktop/Automation tool github/Implementation_Planning/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/jacob_cochran_fws_gov/Documents/Early Detection Monitoring/Implementation_Planning/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B75EAC9-2852-43B1-B438-69C1300C3AEC}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F10D9CD9-FA9E-4BDE-AAF4-9FF0B0A5ECBA}"/>
   <bookViews>
-    <workbookView xWindow="1836" yWindow="3552" windowWidth="22980" windowHeight="11616" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
   </bookViews>
   <sheets>
     <sheet name="metaB_effort" sheetId="1" r:id="rId1"/>
+    <sheet name="Partner_effort" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="39">
   <si>
     <t>Location</t>
   </si>
@@ -1011,22 +1012,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06F6531A-26FC-4EDF-8841-283E7EA69A96}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1062,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1090,7 +1091,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1119,7 +1120,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1148,7 +1149,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1177,7 +1178,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1235,7 +1236,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1261,7 +1262,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1284,7 +1285,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1310,7 +1311,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -1333,7 +1334,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1356,7 +1357,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1382,7 +1383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1405,7 +1406,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1438,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1469,7 +1470,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1495,7 +1496,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1527,7 +1528,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1553,7 +1554,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1585,7 +1586,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1617,7 +1618,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1643,7 +1644,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -1675,7 +1676,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -1707,7 +1708,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1733,7 +1734,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1768,7 +1769,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1797,7 +1798,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -1826,7 +1827,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1875,4 +1876,411 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC37EBF-16D1-450B-BF08-944D0CEFA8CF}">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>42.875659810000002</v>
+      </c>
+      <c r="C2">
+        <v>-78.875949579999997</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3">
+        <v>42.567559340000003</v>
+      </c>
+      <c r="C3">
+        <v>-79.115413599999997</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>94</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4">
+        <v>42.487721780000001</v>
+      </c>
+      <c r="C4">
+        <v>-79.331886679999997</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>76</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5">
+        <v>43.33813</v>
+      </c>
+      <c r="C5">
+        <v>-78.718518000000003</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>42.136245520000003</v>
+      </c>
+      <c r="C6">
+        <v>-80.099798649999997</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7">
+        <v>43.233587</v>
+      </c>
+      <c r="C7">
+        <v>-79.054096999999999</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7">
+        <v>81</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <v>45.002239000000003</v>
+      </c>
+      <c r="C8">
+        <v>-74.792409000000006</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8">
+        <v>124</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>43.035739139999997</v>
+      </c>
+      <c r="C9">
+        <v>-78.842143460000003</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>43.364257000000002</v>
+      </c>
+      <c r="C10">
+        <v>-78.192469000000003</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>84</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>43.463628999999997</v>
+      </c>
+      <c r="C11">
+        <v>-76.520600000000002</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>43.253931999999999</v>
+      </c>
+      <c r="C12">
+        <v>-77.573269999999994</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13">
+        <v>43.569085999999999</v>
+      </c>
+      <c r="C13">
+        <v>-76.203276000000002</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14">
+        <v>43.2648911</v>
+      </c>
+      <c r="C14">
+        <v>-76.98096074</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>57</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15">
+        <v>43.027583540000002</v>
+      </c>
+      <c r="C15">
+        <v>-78.988743009999993</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15">
+        <v>54</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H24">
+    <sortCondition ref="A2:A24"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Numerous updates for 2026 planning
</commit_message>
<xml_diff>
--- a/data/metaB_effort.xlsx
+++ b/data/metaB_effort.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/jacob_cochran_fws_gov/Documents/Early Detection Monitoring/Implementation_Planning/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F10D9CD9-FA9E-4BDE-AAF4-9FF0B0A5ECBA}"/>
+  <xr:revisionPtr revIDLastSave="256" documentId="8_{544D56E2-6810-4C87-AC3D-3B7FD940DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3E78F83-FFD8-4F2C-91DE-7FFE754422EB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{E30D9601-8F6E-4B6E-AA75-88F8C03488F9}"/>
   </bookViews>
   <sheets>
     <sheet name="metaB_effort" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="41">
   <si>
     <t>Location</t>
   </si>
@@ -90,9 +90,6 @@
     <t>North Tonawanda, NY</t>
   </si>
   <si>
-    <t>Moderate</t>
-  </si>
-  <si>
     <t>Upper Niagara River, NY/ON</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
     <t>Cattaragaus Creek, NY</t>
   </si>
   <si>
-    <t>Massena, NY/ON</t>
-  </si>
-  <si>
     <t>Targeted</t>
   </si>
   <si>
@@ -151,6 +145,18 @@
   </si>
   <si>
     <t>Target_Species</t>
+  </si>
+  <si>
+    <t>Black River Bay, NY</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Lake St. Lawrence, NY/ON</t>
+  </si>
+  <si>
+    <t>Lake St. Francis, NY/ON</t>
   </si>
 </sst>
 </file>
@@ -634,8 +640,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1011,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06F6531A-26FC-4EDF-8841-283E7EA69A96}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
@@ -1056,10 +1063,10 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1166,7 +1173,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
         <v>12</v>
@@ -1195,7 +1202,7 @@
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
         <v>12</v>
@@ -1209,7 +1216,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>43.027583540000002</v>
@@ -1224,7 +1231,7 @@
         <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
         <v>12</v>
@@ -1233,12 +1240,12 @@
         <v>20</v>
       </c>
       <c r="I7">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>43.2648911</v>
@@ -1253,18 +1260,15 @@
         <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G8" t="s">
         <v>12</v>
-      </c>
-      <c r="I8">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>44.250826000000004</v>
@@ -1279,15 +1283,21 @@
         <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
+      </c>
+      <c r="H9">
+        <v>30</v>
+      </c>
+      <c r="I9">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>42.487721780000001</v>
@@ -1302,18 +1312,21 @@
         <v>76</v>
       </c>
       <c r="F10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G10" t="s">
         <v>12</v>
       </c>
+      <c r="H10">
+        <v>10</v>
+      </c>
       <c r="I10">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>43.233587</v>
@@ -1328,7 +1341,7 @@
         <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G11" t="s">
         <v>12</v>
@@ -1336,7 +1349,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>43.364257000000002</v>
@@ -1351,7 +1364,7 @@
         <v>84</v>
       </c>
       <c r="F12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G12" t="s">
         <v>12</v>
@@ -1359,7 +1372,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>42.567559340000003</v>
@@ -1374,33 +1387,33 @@
         <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G13" t="s">
         <v>12</v>
       </c>
       <c r="I13">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B14">
-        <v>45.002239000000003</v>
+        <v>44.922373187592399</v>
       </c>
       <c r="C14">
-        <v>-74.792409000000006</v>
+        <v>-75.088118570138903</v>
       </c>
       <c r="D14" t="s">
         <v>14</v>
       </c>
       <c r="E14">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G14" t="s">
         <v>12</v>
@@ -1408,173 +1421,167 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="B15">
-        <v>42.875659810000002</v>
+        <v>44.989308091740398</v>
       </c>
       <c r="C15">
-        <v>-78.875949579999997</v>
+        <v>-74.740341342397102</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E15">
-        <v>3</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15">
-        <v>10</v>
-      </c>
-      <c r="I15">
-        <v>10</v>
-      </c>
-      <c r="K15" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="B16">
-        <v>43.253931999999999</v>
+        <v>43.969969920031197</v>
       </c>
       <c r="C16">
-        <v>-77.573269999999994</v>
+        <v>-76.108388104891603</v>
       </c>
       <c r="D16" t="s">
         <v>14</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="H16">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I16">
-        <v>10</v>
-      </c>
-      <c r="K16" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B17">
-        <v>43.307336999999997</v>
+        <v>42.875659810000002</v>
       </c>
       <c r="C17">
-        <v>-77.717062999999996</v>
+        <v>-78.875949579999997</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="H17">
+        <v>10</v>
+      </c>
+      <c r="I17">
+        <v>10</v>
       </c>
       <c r="K17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B18">
-        <v>43.464136000000003</v>
+        <v>43.253931999999999</v>
       </c>
       <c r="C18">
-        <v>-76.521203</v>
+        <v>-77.573269999999994</v>
       </c>
       <c r="D18" t="s">
         <v>14</v>
       </c>
       <c r="E18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H18">
         <v>10</v>
       </c>
       <c r="I18">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B19">
-        <v>42.136245520000003</v>
+        <v>43.307336999999997</v>
       </c>
       <c r="C19">
-        <v>-80.099798649999997</v>
+        <v>-77.717062999999996</v>
       </c>
       <c r="D19" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E19">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K19" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B20">
-        <v>43.035739139999997</v>
+        <v>43.464136000000003</v>
       </c>
       <c r="C20">
-        <v>-78.842143460000003</v>
+        <v>-76.521203</v>
       </c>
       <c r="D20" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E20">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="G20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H20">
         <v>10</v>
@@ -1583,304 +1590,367 @@
         <v>10</v>
       </c>
       <c r="K20" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B21">
-        <v>43.265535999999997</v>
+        <v>42.136245520000003</v>
       </c>
       <c r="C21">
-        <v>-76.967893000000004</v>
+        <v>-80.099798649999997</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E21">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="F21" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G21" t="s">
-        <v>28</v>
-      </c>
-      <c r="H21">
-        <v>10</v>
-      </c>
-      <c r="I21">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="K21" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B22">
-        <v>42.487721780000001</v>
+        <v>43.035739139999997</v>
       </c>
       <c r="C22">
-        <v>-79.331886679999997</v>
+        <v>-78.842143460000003</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
       <c r="E22">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G22" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="H22">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>30</v>
       </c>
       <c r="K22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B23">
-        <v>43.233587</v>
+        <v>43.265535999999997</v>
       </c>
       <c r="C23">
-        <v>-79.054096999999999</v>
+        <v>-76.967893000000004</v>
       </c>
       <c r="D23" t="s">
         <v>14</v>
       </c>
       <c r="E23">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="F23" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H23">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I23">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K23" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>43.364257000000002</v>
+        <v>42.487721780000001</v>
       </c>
       <c r="C24">
-        <v>-78.192469000000003</v>
+        <v>-79.331886679999997</v>
       </c>
       <c r="D24" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E24">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F24" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="G24" t="s">
-        <v>28</v>
-      </c>
-      <c r="H24">
-        <v>10</v>
-      </c>
-      <c r="I24">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="K24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>43.233587</v>
+      </c>
+      <c r="C25">
+        <v>-79.054096999999999</v>
+      </c>
+      <c r="D25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25">
+        <v>81</v>
+      </c>
+      <c r="F25" t="s">
+        <v>38</v>
+      </c>
+      <c r="G25" t="s">
         <v>26</v>
       </c>
-      <c r="B25">
-        <v>42.567559340000003</v>
-      </c>
-      <c r="C25">
-        <v>-79.115413599999997</v>
-      </c>
-      <c r="D25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25">
-        <v>94</v>
-      </c>
-      <c r="F25" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" t="s">
-        <v>28</v>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="I25">
+        <v>20</v>
       </c>
       <c r="K25" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B26">
-        <v>45.002239000000003</v>
+        <v>43.364257000000002</v>
       </c>
       <c r="C26">
-        <v>-74.792409000000006</v>
+        <v>-78.192469000000003</v>
       </c>
       <c r="D26" t="s">
         <v>14</v>
       </c>
       <c r="E26">
-        <v>124</v>
+        <v>84</v>
       </c>
       <c r="F26" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="G26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H26">
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="I26">
-        <v>110</v>
-      </c>
-      <c r="J26" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="K26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B27">
-        <v>43.33813</v>
+        <v>42.567559340000003</v>
       </c>
       <c r="C27">
-        <v>-78.718518000000003</v>
+        <v>-79.115413599999997</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="E27">
+        <v>94</v>
       </c>
       <c r="F27" t="s">
         <v>11</v>
       </c>
       <c r="G27" t="s">
-        <v>28</v>
-      </c>
-      <c r="H27">
-        <v>10</v>
-      </c>
-      <c r="I27">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="K27" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B28">
-        <v>43.569085999999999</v>
+        <v>44.922373187592399</v>
       </c>
       <c r="C28">
-        <v>-76.203276000000002</v>
+        <v>-75.088118570138903</v>
       </c>
       <c r="D28" t="s">
         <v>14</v>
+      </c>
+      <c r="E28">
+        <v>124</v>
       </c>
       <c r="F28" t="s">
         <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H28">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="I28">
-        <v>20</v>
+        <v>120</v>
+      </c>
+      <c r="J28" t="s">
+        <v>33</v>
       </c>
       <c r="K28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B29">
-        <v>43.300778999999999</v>
+        <v>43.33813</v>
       </c>
       <c r="C29">
-        <v>-76.836208999999997</v>
+        <v>-78.718518000000003</v>
       </c>
       <c r="D29" t="s">
         <v>14</v>
       </c>
+      <c r="E29">
+        <v>118</v>
+      </c>
       <c r="F29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B30">
+        <v>43.569085999999999</v>
+      </c>
+      <c r="C30">
+        <v>-76.203276000000002</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30">
+        <v>107</v>
+      </c>
+      <c r="F30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" t="s">
+        <v>26</v>
+      </c>
+      <c r="K30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>43.300778999999999</v>
+      </c>
+      <c r="C31">
+        <v>-76.836208999999997</v>
+      </c>
+      <c r="D31" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31">
+        <v>210</v>
+      </c>
+      <c r="F31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" t="s">
+        <v>26</v>
+      </c>
+      <c r="K31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
         <v>43.330714999999998</v>
       </c>
-      <c r="C30">
+      <c r="C32">
         <v>-76.705862999999994</v>
       </c>
-      <c r="D30" t="s">
-        <v>14</v>
-      </c>
-      <c r="F30" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" t="s">
-        <v>28</v>
-      </c>
-      <c r="K30" t="s">
-        <v>36</v>
-      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32">
+        <v>116</v>
+      </c>
+      <c r="F32" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" t="s">
+        <v>26</v>
+      </c>
+      <c r="K32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC37EBF-16D1-450B-BF08-944D0CEFA8CF}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
@@ -1947,7 +2017,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3">
         <v>42.567559340000003</v>
@@ -1962,18 +2032,18 @@
         <v>94</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
       <c r="H3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>42.487721780000001</v>
@@ -1988,18 +2058,18 @@
         <v>76</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
       <c r="H4">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5">
         <v>43.33813</v>
@@ -2010,14 +2080,14 @@
       <c r="D5" t="s">
         <v>14</v>
       </c>
+      <c r="E5">
+        <v>118</v>
+      </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2048,7 +2118,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>43.233587</v>
@@ -2063,134 +2133,132 @@
         <v>81</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H7">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B8">
-        <v>45.002239000000003</v>
+        <v>44.922373187592399</v>
       </c>
       <c r="C8">
-        <v>-74.792409000000006</v>
+        <f>--75.0881185701389</f>
+        <v>75.088118570138903</v>
       </c>
       <c r="D8" t="s">
         <v>14</v>
       </c>
       <c r="E8">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H8">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="B9">
-        <v>43.035739139999997</v>
+        <v>44.989308091740398</v>
       </c>
       <c r="C9">
-        <v>-78.842143460000003</v>
+        <v>-74.740341342397102</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
-      </c>
-      <c r="H9">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B10">
-        <v>43.364257000000002</v>
+        <v>43.035739139999997</v>
       </c>
       <c r="C10">
-        <v>-78.192469000000003</v>
+        <v>-78.842143460000003</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="H10">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B11">
-        <v>43.463628999999997</v>
+        <v>43.364257000000002</v>
       </c>
       <c r="C11">
-        <v>-76.520600000000002</v>
+        <v>-78.192469000000003</v>
       </c>
       <c r="D11" t="s">
         <v>14</v>
       </c>
       <c r="E11">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="H11">
-        <v>70</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B12">
-        <v>43.253931999999999</v>
+        <v>43.463628999999997</v>
       </c>
       <c r="C12">
-        <v>-77.573269999999994</v>
+        <v>-76.520600000000002</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" t="s">
         <v>11</v>
@@ -2204,51 +2272,51 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B13">
-        <v>43.569085999999999</v>
+        <v>43.253931999999999</v>
       </c>
       <c r="C13">
-        <v>-76.203276000000002</v>
+        <v>-77.573269999999994</v>
       </c>
       <c r="D13" t="s">
         <v>14</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
       </c>
       <c r="F13" t="s">
         <v>11</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="H13">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B14">
-        <v>43.2648911</v>
+        <v>43.569085999999999</v>
       </c>
       <c r="C14">
-        <v>-76.98096074</v>
+        <v>-76.203276000000002</v>
       </c>
       <c r="D14" t="s">
         <v>14</v>
       </c>
       <c r="E14">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -2256,19 +2324,19 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>43.027583540000002</v>
+        <v>43.2648911</v>
       </c>
       <c r="C15">
-        <v>-78.988743009999993</v>
+        <v>-76.98096074</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E15">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G15" t="s">
         <v>12</v>
@@ -2277,9 +2345,113 @@
         <v>20</v>
       </c>
     </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>43.027583540000002</v>
+      </c>
+      <c r="C16">
+        <v>-78.988743009999993</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16">
+        <v>54</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17">
+        <v>44.250826000000004</v>
+      </c>
+      <c r="C17">
+        <v>-76.087418</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>71</v>
+      </c>
+      <c r="F17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18">
+        <v>44.989308091740398</v>
+      </c>
+      <c r="C18">
+        <v>-74.740341342397102</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18">
+        <v>86</v>
+      </c>
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>43.969969920031197</v>
+      </c>
+      <c r="C19">
+        <v>-76.108388104891603</v>
+      </c>
+      <c r="D19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19">
+        <v>87</v>
+      </c>
+      <c r="F19" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H20" s="1"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H24">
-    <sortCondition ref="A2:A24"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H25">
+    <sortCondition ref="A2:A25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>